<commit_message>
Auto commit at 2026-03-08  8:23:54.35
</commit_message>
<xml_diff>
--- a/data/daydata.xlsx
+++ b/data/daydata.xlsx
@@ -17,7 +17,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="8">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="20" uniqueCount="8">
   <si>
     <t>日期</t>
     <phoneticPr fontId="1" type="noConversion"/>
@@ -405,7 +405,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <sheetPr codeName="Sheet1"/>
-  <dimension ref="A1:J10"/>
+  <dimension ref="A1:J15"/>
   <sheetFormatPr defaultRowHeight="13.5" x14ac:dyDescent="0.15"/>
   <cols>
     <col min="1" max="1" width="12.5" style="1" customWidth="1"/>
@@ -556,8 +556,166 @@
         <v>168</v>
       </c>
     </row>
+    <row r="8" spans="1:10" x14ac:dyDescent="0.15">
+      <c r="A8" s="1">
+        <v>46085</v>
+      </c>
+      <c r="B8" t="s">
+        <v>4</v>
+      </c>
+      <c r="C8" s="3">
+        <v>10307.450000000001</v>
+      </c>
+      <c r="D8" s="3">
+        <v>8932.2000000000007</v>
+      </c>
+      <c r="E8" s="3">
+        <v>3873.42</v>
+      </c>
+      <c r="F8" s="2">
+        <v>422</v>
+      </c>
+    </row>
+    <row r="9" spans="1:10" x14ac:dyDescent="0.15">
+      <c r="A9" s="1">
+        <v>46085</v>
+      </c>
+      <c r="B9" t="s">
+        <v>5</v>
+      </c>
+      <c r="C9" s="3">
+        <v>4210.59</v>
+      </c>
+      <c r="D9" s="3">
+        <v>3594</v>
+      </c>
+      <c r="E9" s="3">
+        <v>1166.73</v>
+      </c>
+      <c r="F9" s="2">
+        <v>155</v>
+      </c>
+    </row>
     <row r="10" spans="1:10" x14ac:dyDescent="0.15">
-      <c r="J10" s="4"/>
+      <c r="A10" s="1">
+        <v>46086</v>
+      </c>
+      <c r="B10" t="s">
+        <v>4</v>
+      </c>
+      <c r="C10" s="3">
+        <v>10181.34</v>
+      </c>
+      <c r="D10" s="3">
+        <v>8583.56</v>
+      </c>
+      <c r="E10" s="3">
+        <v>3822.13</v>
+      </c>
+      <c r="F10" s="2">
+        <v>440</v>
+      </c>
+    </row>
+    <row r="11" spans="1:10" x14ac:dyDescent="0.15">
+      <c r="A11" s="1">
+        <v>46086</v>
+      </c>
+      <c r="B11" t="s">
+        <v>5</v>
+      </c>
+      <c r="C11" s="3">
+        <v>4858.54</v>
+      </c>
+      <c r="D11" s="3">
+        <v>4117.92</v>
+      </c>
+      <c r="E11" s="3">
+        <v>1370.55</v>
+      </c>
+      <c r="F11" s="2">
+        <v>186</v>
+      </c>
+    </row>
+    <row r="12" spans="1:10" x14ac:dyDescent="0.15">
+      <c r="A12" s="1">
+        <v>46087</v>
+      </c>
+      <c r="B12" t="s">
+        <v>4</v>
+      </c>
+      <c r="C12" s="3">
+        <v>9504.34</v>
+      </c>
+      <c r="D12" s="3">
+        <v>8087.71</v>
+      </c>
+      <c r="E12" s="3">
+        <v>3580.41</v>
+      </c>
+      <c r="F12" s="2">
+        <v>427</v>
+      </c>
+    </row>
+    <row r="13" spans="1:10" x14ac:dyDescent="0.15">
+      <c r="A13" s="1">
+        <v>46087</v>
+      </c>
+      <c r="B13" t="s">
+        <v>5</v>
+      </c>
+      <c r="C13" s="3">
+        <v>4402.71</v>
+      </c>
+      <c r="D13" s="3">
+        <v>3740.01</v>
+      </c>
+      <c r="E13" s="3">
+        <v>1196.42</v>
+      </c>
+      <c r="F13" s="2">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="14" spans="1:10" x14ac:dyDescent="0.15">
+      <c r="A14" s="1">
+        <v>46088</v>
+      </c>
+      <c r="B14" t="s">
+        <v>4</v>
+      </c>
+      <c r="C14" s="3">
+        <v>10711.35</v>
+      </c>
+      <c r="D14" s="3">
+        <v>9348.5400000000009</v>
+      </c>
+      <c r="E14" s="3">
+        <v>3942.12</v>
+      </c>
+      <c r="F14" s="2">
+        <v>460</v>
+      </c>
+      <c r="J14" s="4"/>
+    </row>
+    <row r="15" spans="1:10" x14ac:dyDescent="0.15">
+      <c r="A15" s="1">
+        <v>46088</v>
+      </c>
+      <c r="B15" t="s">
+        <v>5</v>
+      </c>
+      <c r="C15" s="3">
+        <v>4449.42</v>
+      </c>
+      <c r="D15" s="3">
+        <v>3668.87</v>
+      </c>
+      <c r="E15" s="3">
+        <v>1290.25</v>
+      </c>
+      <c r="F15" s="2">
+        <v>162</v>
+      </c>
     </row>
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>

</xml_diff>

<commit_message>
Auto commit at 2026-03-12 11:03:06.60
</commit_message>
<xml_diff>
--- a/data/daydata.xlsx
+++ b/data/daydata.xlsx
@@ -17,7 +17,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="20" uniqueCount="8">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="28" uniqueCount="8">
   <si>
     <t>日期</t>
     <phoneticPr fontId="1" type="noConversion"/>
@@ -405,7 +405,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <sheetPr codeName="Sheet1"/>
-  <dimension ref="A1:J15"/>
+  <dimension ref="A1:J23"/>
   <sheetFormatPr defaultRowHeight="13.5" x14ac:dyDescent="0.15"/>
   <cols>
     <col min="1" max="1" width="12.5" style="1" customWidth="1"/>
@@ -717,6 +717,166 @@
         <v>162</v>
       </c>
     </row>
+    <row r="16" spans="1:10" x14ac:dyDescent="0.15">
+      <c r="A16" s="1">
+        <v>46089</v>
+      </c>
+      <c r="B16" t="s">
+        <v>4</v>
+      </c>
+      <c r="C16" s="3">
+        <v>10200.01</v>
+      </c>
+      <c r="D16" s="3">
+        <v>8822.2199999999993</v>
+      </c>
+      <c r="E16" s="3">
+        <v>3758.02</v>
+      </c>
+      <c r="F16" s="2">
+        <v>440</v>
+      </c>
+    </row>
+    <row r="17" spans="1:6" x14ac:dyDescent="0.15">
+      <c r="A17" s="1">
+        <v>46089</v>
+      </c>
+      <c r="B17" t="s">
+        <v>5</v>
+      </c>
+      <c r="C17" s="3">
+        <v>3711</v>
+      </c>
+      <c r="D17" s="3">
+        <v>3148.67</v>
+      </c>
+      <c r="E17" s="3">
+        <v>1011.44</v>
+      </c>
+      <c r="F17" s="2">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="18" spans="1:6" x14ac:dyDescent="0.15">
+      <c r="A18" s="1">
+        <v>46090</v>
+      </c>
+      <c r="B18" t="s">
+        <v>4</v>
+      </c>
+      <c r="C18" s="3">
+        <v>11320.22</v>
+      </c>
+      <c r="D18" s="3">
+        <v>9618.15</v>
+      </c>
+      <c r="E18" s="3">
+        <v>4237.8</v>
+      </c>
+      <c r="F18" s="2">
+        <v>483</v>
+      </c>
+    </row>
+    <row r="19" spans="1:6" x14ac:dyDescent="0.15">
+      <c r="A19" s="1">
+        <v>46090</v>
+      </c>
+      <c r="B19" t="s">
+        <v>5</v>
+      </c>
+      <c r="C19" s="3">
+        <v>5512.38</v>
+      </c>
+      <c r="D19" s="3">
+        <v>4756.82</v>
+      </c>
+      <c r="E19" s="3">
+        <v>1502.97</v>
+      </c>
+      <c r="F19" s="2">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="20" spans="1:6" x14ac:dyDescent="0.15">
+      <c r="A20" s="1">
+        <v>46091</v>
+      </c>
+      <c r="B20" t="s">
+        <v>4</v>
+      </c>
+      <c r="C20" s="3">
+        <v>10379.68</v>
+      </c>
+      <c r="D20" s="3">
+        <v>8926.42</v>
+      </c>
+      <c r="E20" s="3">
+        <v>3917.06</v>
+      </c>
+      <c r="F20" s="2">
+        <v>441</v>
+      </c>
+    </row>
+    <row r="21" spans="1:6" x14ac:dyDescent="0.15">
+      <c r="A21" s="1">
+        <v>46091</v>
+      </c>
+      <c r="B21" t="s">
+        <v>5</v>
+      </c>
+      <c r="C21" s="3">
+        <v>5059.08</v>
+      </c>
+      <c r="D21" s="3">
+        <v>4324.0600000000004</v>
+      </c>
+      <c r="E21" s="3">
+        <v>1392.88</v>
+      </c>
+      <c r="F21" s="2">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="22" spans="1:6" x14ac:dyDescent="0.15">
+      <c r="A22" s="1">
+        <v>46092</v>
+      </c>
+      <c r="B22" t="s">
+        <v>4</v>
+      </c>
+      <c r="C22" s="3">
+        <v>9668.66</v>
+      </c>
+      <c r="D22" s="3">
+        <v>8242.83</v>
+      </c>
+      <c r="E22" s="3">
+        <v>3618.74</v>
+      </c>
+      <c r="F22" s="2">
+        <v>438</v>
+      </c>
+    </row>
+    <row r="23" spans="1:6" x14ac:dyDescent="0.15">
+      <c r="A23" s="1">
+        <v>46092</v>
+      </c>
+      <c r="B23" t="s">
+        <v>5</v>
+      </c>
+      <c r="C23" s="3">
+        <v>4401.9399999999996</v>
+      </c>
+      <c r="D23" s="3">
+        <v>3810.49</v>
+      </c>
+      <c r="E23" s="3">
+        <v>1250.73</v>
+      </c>
+      <c r="F23" s="2">
+        <v>164</v>
+      </c>
+    </row>
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>